<commit_message>
pretty good actually [ euphoria v1]
</commit_message>
<xml_diff>
--- a/docs/DECISIONS.xlsx
+++ b/docs/DECISIONS.xlsx
@@ -3838,7 +3838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="13" min="1" max="1"/>
@@ -4074,6 +4074,116 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Price-assisted END gate (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>PASSED all pre-stated conditions: G2 boom thresholds as a live prerequisite -&gt; capture 16-&gt;26 detectable tops (matched years), AP 0.286-&gt;0.435, FAs 44-&gt;41, capture-gain CI [+3.5pp,+13pp]. Offered as labelled second signal; claim becomes 'crowd + chart'.</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>The gate reuses the ground-truth boom definition on trailing prices - no new constant, no look-ahead.</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>NB03 commissioned-test section</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Combined price+crowd ALERT bank (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>REJECTED under pre-stated criterion: 65% cliff-30 hit rate indistinguishable from its own 62% candidate-day baseline (CI includes 0). Smoothed-trigger evidence retained: FA 31-&gt;24 at equal capture, median trigger run 6-&gt;8d.</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>The alert layer cannot out-predict its own danger state; its job is timing the peak, which it does (median 8d lead).</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>NB06 desk-signal study</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>DANGER STATE shipped (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>The candidacy state (A1 2x hype AND G2 boom) validated as the standing drop-warning: cliff-30 = 62% in-state vs 19% ordinary, uplift CI [+28pp,+50pp]. Rendered as the amber band on every terminal price panel.</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Pure composition of two existing constants; the single most actionable statistic of the project for the PM use case.</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>NB06; dashboard danger band; PARAMETER_REGISTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>DESK CONFIGURATION adopted: GET OUT (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>Boom-gated END rules + 7d-smoothed (ROLL) trigger. Walk-forward: capture 24/122 detectable tops, FA 39 (0.195/instr-yr), AP 0.449 (raw gate 0.435), median warning 8d before the peak. Smoothing adopted by pre-stated rule (AP not lower AND FAs not higher); 2-capture cost recorded. Frozen live threshold 0.630 (budget rule, full prior years).</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>The desk lifted the crowd-only rule for a labelled SECOND family ('use both price and social media - I want a better hit rate') and demanded no one-day blips. Candidacy = A1 hype AND G2 boom (existing constants only).</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>NB06 adopted-configuration section; euphoria_desk_report.json; euphoria_phases.py §6</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>DESK CONFIGURATION adopted: GET IN (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Phase-aware onset (end-stage days - A1∧A2∧A3-persistence - excluded from candidacy) + 7d smoothing. Adjacency (START within 21d before an END) 20→2, LATE 21→10, FA 169→124; capture cost 29→20 of 125 RECORDED. Frozen live threshold 0.848. OVERRULES the earlier utility-rule rejection of the phase-aware variant as an explicit desk decision.</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>The desk stated three times that a START landing on an END destroys PM trust - adjacency is the binding constraint, so it overrules raw capture. Selection rule pre-stated in NB06; drift guard pins notebook == production.</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
+        <is>
+          <t>NB06; euphoria_desk_report.json; PARAMETER_REGISTER class 5; dashboard GET IN/GET OUT banners</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>